<commit_message>
data: manual transcript fixes (074f2ec, 0a48c888, 151f2ec) + rebuild db + xlsx checklist update
</commit_message>
<xml_diff>
--- a/data/s1/transcripts_index.xlsx
+++ b/data/s1/transcripts_index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abyos\Documents\GitHub\Haparlamentor\data\s1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860A3E85-E81D-4342-A724-E2D8BAB3302F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B6211D-9A10-49CE-9676-EB1D898DD7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="85">
   <si>
     <t>#</t>
   </si>
@@ -752,6 +752,9 @@
       <c r="F4" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="G4" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
@@ -772,6 +775,9 @@
       <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="G5" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
@@ -791,6 +797,9 @@
       </c>
       <c r="F6" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
feat(footer): BMC support link with thanks toast + drop broken short
- Footer: add centered "קנה לי קפה" link with Coffee icon (placeholder
  href="#" until BMC account is set up). Click shows a 3.5s "תודה רבה"
  toast (framer-motion) while opening BMC in a new tab.
- Data: remove "אמציה ושאולי במונית - נפל בעריכה" short (no usable
  content), delete its transcript, rebuild db.json (37→36 shorts).
- Transcripts: pull in manual fixes for 3579a54e and 3641fef1.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/s1/transcripts_index.xlsx
+++ b/data/s1/transcripts_index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abyos\Documents\GitHub\Haparlamentor\data\s1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B6211D-9A10-49CE-9676-EB1D898DD7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCA635C-4AC5-48E1-B9D0-F5F6411E080A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5070" yWindow="5070" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="S1 Transcripts" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="87">
   <si>
     <t>#</t>
   </si>
@@ -283,6 +283,12 @@
   </si>
   <si>
     <t>בוצע</t>
+  </si>
+  <si>
+    <t>ירד</t>
+  </si>
+  <si>
+    <t>ללא קול</t>
   </si>
 </sst>
 </file>
@@ -821,6 +827,9 @@
       <c r="F7" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="G7" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
@@ -841,6 +850,9 @@
       <c r="F8" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="G8" s="3" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
@@ -860,6 +872,9 @@
       </c>
       <c r="F9" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="G9" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>